<commit_message>
AicsTracker dashboard from AICS
</commit_message>
<xml_diff>
--- a/AicsTracker/AicsGlobal_Classifications_TimeWindows.xlsx
+++ b/AicsTracker/AicsGlobal_Classifications_TimeWindows.xlsx
@@ -1067,7 +1067,7 @@
         <v>46204.815416666665</v>
       </c>
       <c r="F2" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G2" s="0" t="s">
         <v>24</v>
@@ -1076,7 +1076,7 @@
         <v>24</v>
       </c>
       <c r="I2" s="0" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="J2" s="0" t="s">
         <v>25</v>
@@ -1096,8 +1096,8 @@
       <c r="O2" s="0">
         <v>0</v>
       </c>
-      <c r="P2" s="0" t="s">
-        <v>25</v>
+      <c r="P2" s="0">
+        <v>1</v>
       </c>
       <c r="Q2" s="0" t="s">
         <v>25</v>
@@ -1135,7 +1135,7 @@
         <v>46204.34583333333</v>
       </c>
       <c r="F3" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G3" s="0" t="s">
         <v>28</v>
@@ -1203,7 +1203,7 @@
         <v>46207.15827546296</v>
       </c>
       <c r="F4" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G4" s="0" t="s">
         <v>28</v>
@@ -1215,7 +1215,7 @@
         <v>28</v>
       </c>
       <c r="J4" s="0" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="K4" s="0" t="s">
         <v>25</v>
@@ -1235,8 +1235,8 @@
       <c r="P4" s="0">
         <v>0</v>
       </c>
-      <c r="Q4" s="0" t="s">
-        <v>25</v>
+      <c r="Q4" s="0">
+        <v>0</v>
       </c>
       <c r="R4" s="0" t="s">
         <v>25</v>
@@ -1271,7 +1271,7 @@
         <v>46204.81548611111</v>
       </c>
       <c r="F5" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G5" s="0" t="s">
         <v>24</v>
@@ -1280,7 +1280,7 @@
         <v>24</v>
       </c>
       <c r="I5" s="0" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="J5" s="0" t="s">
         <v>25</v>
@@ -1300,8 +1300,8 @@
       <c r="O5" s="0">
         <v>0</v>
       </c>
-      <c r="P5" s="0" t="s">
-        <v>25</v>
+      <c r="P5" s="0">
+        <v>1</v>
       </c>
       <c r="Q5" s="0" t="s">
         <v>25</v>
@@ -1339,7 +1339,7 @@
         <v>46200.30415509259</v>
       </c>
       <c r="F6" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G6" s="0" t="s">
         <v>28</v>
@@ -1407,7 +1407,7 @@
         <v>46214.27086805556</v>
       </c>
       <c r="F7" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G7" s="0" t="s">
         <v>28</v>
@@ -1475,7 +1475,7 @@
         <v>46196.08100694444</v>
       </c>
       <c r="F8" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G8" s="0" t="s">
         <v>24</v>
@@ -1543,7 +1543,7 @@
         <v>46211.80736111111</v>
       </c>
       <c r="F9" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G9" s="0" t="s">
         <v>28</v>
@@ -1552,7 +1552,7 @@
         <v>28</v>
       </c>
       <c r="I9" s="0" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="J9" s="0" t="s">
         <v>25</v>
@@ -1572,8 +1572,8 @@
       <c r="O9" s="0">
         <v>0</v>
       </c>
-      <c r="P9" s="0" t="s">
-        <v>25</v>
+      <c r="P9" s="0">
+        <v>0</v>
       </c>
       <c r="Q9" s="0" t="s">
         <v>25</v>
@@ -1611,7 +1611,7 @@
         <v>46214.30170138889</v>
       </c>
       <c r="F10" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G10" s="0" t="s">
         <v>24</v>
@@ -1679,7 +1679,7 @@
         <v>46211.689108796294</v>
       </c>
       <c r="F11" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G11" s="0" t="s">
         <v>28</v>
@@ -1688,7 +1688,7 @@
         <v>28</v>
       </c>
       <c r="I11" s="0" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="J11" s="0" t="s">
         <v>25</v>
@@ -1708,8 +1708,8 @@
       <c r="O11" s="0">
         <v>1</v>
       </c>
-      <c r="P11" s="0" t="s">
-        <v>25</v>
+      <c r="P11" s="0">
+        <v>0</v>
       </c>
       <c r="Q11" s="0" t="s">
         <v>25</v>
@@ -1747,7 +1747,7 @@
         <v>46198.75680555555</v>
       </c>
       <c r="F12" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G12" s="0" t="s">
         <v>24</v>
@@ -1759,7 +1759,7 @@
         <v>24</v>
       </c>
       <c r="J12" s="0" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="K12" s="0" t="s">
         <v>25</v>
@@ -1779,8 +1779,8 @@
       <c r="P12" s="0">
         <v>1</v>
       </c>
-      <c r="Q12" s="0" t="s">
-        <v>25</v>
+      <c r="Q12" s="0">
+        <v>0</v>
       </c>
       <c r="R12" s="0" t="s">
         <v>25</v>
@@ -1815,7 +1815,7 @@
         <v>46200.02773148148</v>
       </c>
       <c r="F13" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G13" s="0" t="s">
         <v>28</v>
@@ -1883,7 +1883,7 @@
         <v>46200.57623842593</v>
       </c>
       <c r="F14" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G14" s="0" t="s">
         <v>28</v>
@@ -1951,7 +1951,7 @@
         <v>46198.764027777775</v>
       </c>
       <c r="F15" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G15" s="0" t="s">
         <v>24</v>
@@ -1963,7 +1963,7 @@
         <v>24</v>
       </c>
       <c r="J15" s="0" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="K15" s="0" t="s">
         <v>25</v>
@@ -1983,8 +1983,8 @@
       <c r="P15" s="0">
         <v>1</v>
       </c>
-      <c r="Q15" s="0" t="s">
-        <v>25</v>
+      <c r="Q15" s="0">
+        <v>0</v>
       </c>
       <c r="R15" s="0" t="s">
         <v>25</v>
@@ -2019,7 +2019,7 @@
         <v>46198.18491898148</v>
       </c>
       <c r="F16" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G16" s="0" t="s">
         <v>28</v>
@@ -2087,7 +2087,7 @@
         <v>46203.81460648148</v>
       </c>
       <c r="F17" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G17" s="0" t="s">
         <v>45</v>
@@ -2155,7 +2155,7 @@
         <v>46201.33733796296</v>
       </c>
       <c r="F18" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G18" s="0" t="s">
         <v>28</v>
@@ -2191,7 +2191,7 @@
         <v>0</v>
       </c>
       <c r="R18" s="0">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S18" s="0" t="s">
         <v>25</v>
@@ -2223,7 +2223,7 @@
         <v>46203.71907407408</v>
       </c>
       <c r="F19" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G19" s="0" t="s">
         <v>28</v>
@@ -2291,7 +2291,7 @@
         <v>46195.59105324074</v>
       </c>
       <c r="F20" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G20" s="0" t="s">
         <v>24</v>
@@ -2359,7 +2359,7 @@
         <v>46201.06361111111</v>
       </c>
       <c r="F21" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G21" s="0" t="s">
         <v>28</v>
@@ -2374,7 +2374,7 @@
         <v>28</v>
       </c>
       <c r="K21" s="0" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="L21" s="0" t="s">
         <v>25</v>
@@ -2394,8 +2394,8 @@
       <c r="Q21" s="0">
         <v>1</v>
       </c>
-      <c r="R21" s="0" t="s">
-        <v>25</v>
+      <c r="R21" s="0">
+        <v>0</v>
       </c>
       <c r="S21" s="0" t="s">
         <v>25</v>
@@ -2427,7 +2427,7 @@
         <v>46195.68219907407</v>
       </c>
       <c r="F22" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G22" s="0" t="s">
         <v>24</v>
@@ -2454,7 +2454,7 @@
         <v>25</v>
       </c>
       <c r="O22" s="0">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P22" s="0" t="s">
         <v>25</v>
@@ -2495,7 +2495,7 @@
         <v>46197.83574074074</v>
       </c>
       <c r="F23" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G23" s="0" t="s">
         <v>24</v>
@@ -2563,7 +2563,7 @@
         <v>46198.5140625</v>
       </c>
       <c r="F24" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G24" s="0" t="s">
         <v>24</v>
@@ -2631,7 +2631,7 @@
         <v>46209.61792824074</v>
       </c>
       <c r="F25" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G25" s="0" t="s">
         <v>45</v>
@@ -2699,7 +2699,7 @@
         <v>46202.38591435185</v>
       </c>
       <c r="F26" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G26" s="0" t="s">
         <v>28</v>
@@ -2714,7 +2714,7 @@
         <v>28</v>
       </c>
       <c r="K26" s="0" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="L26" s="0" t="s">
         <v>25</v>
@@ -2734,8 +2734,8 @@
       <c r="Q26" s="0">
         <v>0</v>
       </c>
-      <c r="R26" s="0" t="s">
-        <v>25</v>
+      <c r="R26" s="0">
+        <v>0</v>
       </c>
       <c r="S26" s="0" t="s">
         <v>25</v>
@@ -2767,7 +2767,7 @@
         <v>46215.03915509259</v>
       </c>
       <c r="F27" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G27" s="0" t="s">
         <v>45</v>
@@ -2835,7 +2835,7 @@
         <v>46203.665925925925</v>
       </c>
       <c r="F28" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G28" s="0" t="s">
         <v>24</v>
@@ -2847,7 +2847,7 @@
         <v>24</v>
       </c>
       <c r="J28" s="0" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="K28" s="0" t="s">
         <v>25</v>
@@ -2867,8 +2867,8 @@
       <c r="P28" s="0">
         <v>1</v>
       </c>
-      <c r="Q28" s="0" t="s">
-        <v>25</v>
+      <c r="Q28" s="0">
+        <v>0</v>
       </c>
       <c r="R28" s="0" t="s">
         <v>25</v>
@@ -2903,7 +2903,7 @@
         <v>46205.25707175926</v>
       </c>
       <c r="F29" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G29" s="0" t="s">
         <v>28</v>
@@ -2971,7 +2971,7 @@
         <v>46203.77983796296</v>
       </c>
       <c r="F30" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G30" s="0" t="s">
         <v>45</v>
@@ -3039,7 +3039,7 @@
         <v>46207.957766203705</v>
       </c>
       <c r="F31" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G31" s="0" t="s">
         <v>45</v>
@@ -3107,7 +3107,7 @@
         <v>46204.23569444445</v>
       </c>
       <c r="F32" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G32" s="0" t="s">
         <v>28</v>
@@ -3175,7 +3175,7 @@
         <v>46206.293020833335</v>
       </c>
       <c r="F33" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G33" s="0" t="s">
         <v>45</v>
@@ -3243,7 +3243,7 @@
         <v>46214.75530092593</v>
       </c>
       <c r="F34" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G34" s="0" t="s">
         <v>45</v>
@@ -3311,7 +3311,7 @@
         <v>46198.763715277775</v>
       </c>
       <c r="F35" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G35" s="0" t="s">
         <v>24</v>
@@ -3323,7 +3323,7 @@
         <v>24</v>
       </c>
       <c r="J35" s="0" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="K35" s="0" t="s">
         <v>25</v>
@@ -3343,8 +3343,8 @@
       <c r="P35" s="0">
         <v>1</v>
       </c>
-      <c r="Q35" s="0" t="s">
-        <v>25</v>
+      <c r="Q35" s="0">
+        <v>0</v>
       </c>
       <c r="R35" s="0" t="s">
         <v>25</v>
@@ -3379,7 +3379,7 @@
         <v>46205.502962962964</v>
       </c>
       <c r="F36" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G36" s="0" t="s">
         <v>28</v>
@@ -3391,7 +3391,7 @@
         <v>28</v>
       </c>
       <c r="J36" s="0" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="K36" s="0" t="s">
         <v>25</v>
@@ -3411,8 +3411,8 @@
       <c r="P36" s="0">
         <v>0</v>
       </c>
-      <c r="Q36" s="0" t="s">
-        <v>25</v>
+      <c r="Q36" s="0">
+        <v>0</v>
       </c>
       <c r="R36" s="0" t="s">
         <v>25</v>
@@ -3447,7 +3447,7 @@
         <v>46214.35975694445</v>
       </c>
       <c r="F37" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G37" s="0" t="s">
         <v>28</v>
@@ -3474,7 +3474,7 @@
         <v>25</v>
       </c>
       <c r="O37" s="0">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P37" s="0" t="s">
         <v>25</v>
@@ -3515,7 +3515,7 @@
         <v>46200.67046296296</v>
       </c>
       <c r="F38" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G38" s="0" t="s">
         <v>24</v>
@@ -3583,7 +3583,7 @@
         <v>46215.29809027778</v>
       </c>
       <c r="F39" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G39" s="0" t="s">
         <v>28</v>
@@ -3651,7 +3651,7 @@
         <v>46204.81548611111</v>
       </c>
       <c r="F40" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G40" s="0" t="s">
         <v>24</v>
@@ -3660,7 +3660,7 @@
         <v>24</v>
       </c>
       <c r="I40" s="0" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="J40" s="0" t="s">
         <v>25</v>
@@ -3680,8 +3680,8 @@
       <c r="O40" s="0">
         <v>0</v>
       </c>
-      <c r="P40" s="0" t="s">
-        <v>25</v>
+      <c r="P40" s="0">
+        <v>1</v>
       </c>
       <c r="Q40" s="0" t="s">
         <v>25</v>
@@ -3719,7 +3719,7 @@
         <v>46207.76193287037</v>
       </c>
       <c r="F41" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G41" s="0" t="s">
         <v>24</v>
@@ -3728,7 +3728,7 @@
         <v>24</v>
       </c>
       <c r="I41" s="0" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="J41" s="0" t="s">
         <v>25</v>
@@ -3748,8 +3748,8 @@
       <c r="O41" s="0">
         <v>1</v>
       </c>
-      <c r="P41" s="0" t="s">
-        <v>25</v>
+      <c r="P41" s="0">
+        <v>0</v>
       </c>
       <c r="Q41" s="0" t="s">
         <v>25</v>
@@ -3787,7 +3787,7 @@
         <v>46199.574282407404</v>
       </c>
       <c r="F42" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G42" s="0" t="s">
         <v>28</v>
@@ -3855,7 +3855,7 @@
         <v>46198.758518518516</v>
       </c>
       <c r="F43" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G43" s="0" t="s">
         <v>24</v>
@@ -3867,7 +3867,7 @@
         <v>24</v>
       </c>
       <c r="J43" s="0" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="K43" s="0" t="s">
         <v>25</v>
@@ -3887,8 +3887,8 @@
       <c r="P43" s="0">
         <v>1</v>
       </c>
-      <c r="Q43" s="0" t="s">
-        <v>25</v>
+      <c r="Q43" s="0">
+        <v>0</v>
       </c>
       <c r="R43" s="0" t="s">
         <v>25</v>
@@ -3923,7 +3923,7 @@
         <v>46199.20893518518</v>
       </c>
       <c r="F44" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G44" s="0" t="s">
         <v>28</v>
@@ -3991,7 +3991,7 @@
         <v>46198.76384259259</v>
       </c>
       <c r="F45" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G45" s="0" t="s">
         <v>24</v>
@@ -4003,7 +4003,7 @@
         <v>24</v>
       </c>
       <c r="J45" s="0" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="K45" s="0" t="s">
         <v>25</v>
@@ -4023,8 +4023,8 @@
       <c r="P45" s="0">
         <v>1</v>
       </c>
-      <c r="Q45" s="0" t="s">
-        <v>25</v>
+      <c r="Q45" s="0">
+        <v>0</v>
       </c>
       <c r="R45" s="0" t="s">
         <v>25</v>
@@ -4059,7 +4059,7 @@
         <v>46207.98546296296</v>
       </c>
       <c r="F46" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G46" s="0" t="s">
         <v>28</v>
@@ -4127,7 +4127,7 @@
         <v>46198.758414351854</v>
       </c>
       <c r="F47" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G47" s="0" t="s">
         <v>24</v>
@@ -4139,7 +4139,7 @@
         <v>24</v>
       </c>
       <c r="J47" s="0" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="K47" s="0" t="s">
         <v>25</v>
@@ -4159,8 +4159,8 @@
       <c r="P47" s="0">
         <v>1</v>
       </c>
-      <c r="Q47" s="0" t="s">
-        <v>25</v>
+      <c r="Q47" s="0">
+        <v>0</v>
       </c>
       <c r="R47" s="0" t="s">
         <v>25</v>
@@ -4195,7 +4195,7 @@
         <v>46207.95777777778</v>
       </c>
       <c r="F48" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G48" s="0" t="s">
         <v>24</v>
@@ -4263,7 +4263,7 @@
         <v>46213.479849537034</v>
       </c>
       <c r="F49" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G49" s="0" t="s">
         <v>28</v>
@@ -4290,7 +4290,7 @@
         <v>25</v>
       </c>
       <c r="O49" s="0">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P49" s="0" t="s">
         <v>25</v>
@@ -4331,7 +4331,7 @@
         <v>46213.89649305555</v>
       </c>
       <c r="F50" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G50" s="0" t="s">
         <v>28</v>
@@ -4399,7 +4399,7 @@
         <v>46194.2578587963</v>
       </c>
       <c r="F51" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G51" s="0" t="s">
         <v>28</v>
@@ -4435,7 +4435,7 @@
         <v>1</v>
       </c>
       <c r="R51" s="0">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S51" s="0" t="s">
         <v>25</v>
@@ -4467,7 +4467,7 @@
         <v>46197.83574074074</v>
       </c>
       <c r="F52" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G52" s="0" t="s">
         <v>24</v>
@@ -4535,7 +4535,7 @@
         <v>46214.741215277776</v>
       </c>
       <c r="F53" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G53" s="0" t="s">
         <v>28</v>
@@ -4603,7 +4603,7 @@
         <v>46204.816157407404</v>
       </c>
       <c r="F54" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G54" s="0" t="s">
         <v>24</v>
@@ -4612,7 +4612,7 @@
         <v>24</v>
       </c>
       <c r="I54" s="0" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="J54" s="0" t="s">
         <v>25</v>
@@ -4632,8 +4632,8 @@
       <c r="O54" s="0">
         <v>0</v>
       </c>
-      <c r="P54" s="0" t="s">
-        <v>25</v>
+      <c r="P54" s="0">
+        <v>1</v>
       </c>
       <c r="Q54" s="0" t="s">
         <v>25</v>
@@ -4671,7 +4671,7 @@
         <v>46210.94122685185</v>
       </c>
       <c r="F55" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G55" s="0" t="s">
         <v>28</v>
@@ -4739,7 +4739,7 @@
         <v>46211.91608796296</v>
       </c>
       <c r="F56" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G56" s="0" t="s">
         <v>28</v>
@@ -4748,7 +4748,7 @@
         <v>28</v>
       </c>
       <c r="I56" s="0" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="J56" s="0" t="s">
         <v>25</v>
@@ -4768,8 +4768,8 @@
       <c r="O56" s="0">
         <v>1</v>
       </c>
-      <c r="P56" s="0" t="s">
-        <v>25</v>
+      <c r="P56" s="0">
+        <v>0</v>
       </c>
       <c r="Q56" s="0" t="s">
         <v>25</v>
@@ -4807,7 +4807,7 @@
         <v>46211.9408912037</v>
       </c>
       <c r="F57" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G57" s="0" t="s">
         <v>28</v>
@@ -4816,7 +4816,7 @@
         <v>28</v>
       </c>
       <c r="I57" s="0" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="J57" s="0" t="s">
         <v>25</v>
@@ -4836,8 +4836,8 @@
       <c r="O57" s="0">
         <v>0</v>
       </c>
-      <c r="P57" s="0" t="s">
-        <v>25</v>
+      <c r="P57" s="0">
+        <v>0</v>
       </c>
       <c r="Q57" s="0" t="s">
         <v>25</v>
@@ -4875,7 +4875,7 @@
         <v>46198.763449074075</v>
       </c>
       <c r="F58" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G58" s="0" t="s">
         <v>24</v>
@@ -4887,7 +4887,7 @@
         <v>24</v>
       </c>
       <c r="J58" s="0" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="K58" s="0" t="s">
         <v>25</v>
@@ -4907,8 +4907,8 @@
       <c r="P58" s="0">
         <v>1</v>
       </c>
-      <c r="Q58" s="0" t="s">
-        <v>25</v>
+      <c r="Q58" s="0">
+        <v>0</v>
       </c>
       <c r="R58" s="0" t="s">
         <v>25</v>
@@ -4943,7 +4943,7 @@
         <v>46198.758125</v>
       </c>
       <c r="F59" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G59" s="0" t="s">
         <v>24</v>
@@ -4955,7 +4955,7 @@
         <v>24</v>
       </c>
       <c r="J59" s="0" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="K59" s="0" t="s">
         <v>25</v>
@@ -4975,8 +4975,8 @@
       <c r="P59" s="0">
         <v>1</v>
       </c>
-      <c r="Q59" s="0" t="s">
-        <v>25</v>
+      <c r="Q59" s="0">
+        <v>0</v>
       </c>
       <c r="R59" s="0" t="s">
         <v>25</v>
@@ -5011,7 +5011,7 @@
         <v>46201.54498842593</v>
       </c>
       <c r="F60" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G60" s="0" t="s">
         <v>28</v>
@@ -5026,7 +5026,7 @@
         <v>28</v>
       </c>
       <c r="K60" s="0" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="L60" s="0" t="s">
         <v>25</v>
@@ -5046,8 +5046,8 @@
       <c r="Q60" s="0">
         <v>0</v>
       </c>
-      <c r="R60" s="0" t="s">
-        <v>25</v>
+      <c r="R60" s="0">
+        <v>0</v>
       </c>
       <c r="S60" s="0" t="s">
         <v>25</v>
@@ -5079,7 +5079,7 @@
         <v>46198.76478009259</v>
       </c>
       <c r="F61" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G61" s="0" t="s">
         <v>24</v>
@@ -5091,7 +5091,7 @@
         <v>24</v>
       </c>
       <c r="J61" s="0" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="K61" s="0" t="s">
         <v>25</v>
@@ -5111,8 +5111,8 @@
       <c r="P61" s="0">
         <v>1</v>
       </c>
-      <c r="Q61" s="0" t="s">
-        <v>25</v>
+      <c r="Q61" s="0">
+        <v>0</v>
       </c>
       <c r="R61" s="0" t="s">
         <v>25</v>
@@ -5147,7 +5147,7 @@
         <v>46205.76315972222</v>
       </c>
       <c r="F62" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G62" s="0" t="s">
         <v>28</v>
@@ -5215,7 +5215,7 @@
         <v>46204.83986111111</v>
       </c>
       <c r="F63" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G63" s="0" t="s">
         <v>28</v>
@@ -5283,7 +5283,7 @@
         <v>46203.69975694444</v>
       </c>
       <c r="F64" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G64" s="0" t="s">
         <v>45</v>
@@ -5351,7 +5351,7 @@
         <v>46204.815405092595</v>
       </c>
       <c r="F65" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G65" s="0" t="s">
         <v>24</v>
@@ -5360,7 +5360,7 @@
         <v>24</v>
       </c>
       <c r="I65" s="0" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="J65" s="0" t="s">
         <v>25</v>
@@ -5380,8 +5380,8 @@
       <c r="O65" s="0">
         <v>0</v>
       </c>
-      <c r="P65" s="0" t="s">
-        <v>25</v>
+      <c r="P65" s="0">
+        <v>1</v>
       </c>
       <c r="Q65" s="0" t="s">
         <v>25</v>
@@ -5419,7 +5419,7 @@
         <v>46208.10663194444</v>
       </c>
       <c r="F66" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G66" s="0" t="s">
         <v>28</v>
@@ -5487,7 +5487,7 @@
         <v>46200.854166666664</v>
       </c>
       <c r="F67" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G67" s="0" t="s">
         <v>24</v>
@@ -5555,7 +5555,7 @@
         <v>46204.815416666665</v>
       </c>
       <c r="F68" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G68" s="0" t="s">
         <v>24</v>
@@ -5564,7 +5564,7 @@
         <v>24</v>
       </c>
       <c r="I68" s="0" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="J68" s="0" t="s">
         <v>25</v>
@@ -5584,8 +5584,8 @@
       <c r="O68" s="0">
         <v>0</v>
       </c>
-      <c r="P68" s="0" t="s">
-        <v>25</v>
+      <c r="P68" s="0">
+        <v>1</v>
       </c>
       <c r="Q68" s="0" t="s">
         <v>25</v>
@@ -5623,7 +5623,7 @@
         <v>46205.07099537037</v>
       </c>
       <c r="F69" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G69" s="0" t="s">
         <v>24</v>
@@ -5691,7 +5691,7 @@
         <v>46204.145219907405</v>
       </c>
       <c r="F70" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G70" s="0" t="s">
         <v>24</v>
@@ -5703,7 +5703,7 @@
         <v>24</v>
       </c>
       <c r="J70" s="0" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="K70" s="0" t="s">
         <v>25</v>
@@ -5723,8 +5723,8 @@
       <c r="P70" s="0">
         <v>1</v>
       </c>
-      <c r="Q70" s="0" t="s">
-        <v>25</v>
+      <c r="Q70" s="0">
+        <v>0</v>
       </c>
       <c r="R70" s="0" t="s">
         <v>25</v>
@@ -5759,7 +5759,7 @@
         <v>46191.31182870371</v>
       </c>
       <c r="F71" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G71" s="0" t="s">
         <v>24</v>
@@ -5827,7 +5827,7 @@
         <v>46199.29518518518</v>
       </c>
       <c r="F72" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G72" s="0" t="s">
         <v>28</v>
@@ -5895,7 +5895,7 @@
         <v>46184.345671296294</v>
       </c>
       <c r="F73" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G73" s="0" t="s">
         <v>24</v>
@@ -5904,7 +5904,7 @@
         <v>24</v>
       </c>
       <c r="I73" s="0" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="J73" s="0" t="s">
         <v>25</v>
@@ -5924,8 +5924,8 @@
       <c r="O73" s="0">
         <v>1</v>
       </c>
-      <c r="P73" s="0" t="s">
-        <v>25</v>
+      <c r="P73" s="0">
+        <v>0</v>
       </c>
       <c r="Q73" s="0" t="s">
         <v>25</v>
@@ -5963,7 +5963,7 @@
         <v>46215.31277777778</v>
       </c>
       <c r="F74" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G74" s="0" t="s">
         <v>28</v>
@@ -6031,7 +6031,7 @@
         <v>46198.758576388886</v>
       </c>
       <c r="F75" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G75" s="0" t="s">
         <v>24</v>
@@ -6043,7 +6043,7 @@
         <v>24</v>
       </c>
       <c r="J75" s="0" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="K75" s="0" t="s">
         <v>25</v>
@@ -6063,8 +6063,8 @@
       <c r="P75" s="0">
         <v>1</v>
       </c>
-      <c r="Q75" s="0" t="s">
-        <v>25</v>
+      <c r="Q75" s="0">
+        <v>0</v>
       </c>
       <c r="R75" s="0" t="s">
         <v>25</v>
@@ -6099,7 +6099,7 @@
         <v>46211.747719907406</v>
       </c>
       <c r="F76" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G76" s="0" t="s">
         <v>24</v>
@@ -6108,7 +6108,7 @@
         <v>24</v>
       </c>
       <c r="I76" s="0" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="J76" s="0" t="s">
         <v>25</v>
@@ -6128,8 +6128,8 @@
       <c r="O76" s="0">
         <v>0</v>
       </c>
-      <c r="P76" s="0" t="s">
-        <v>25</v>
+      <c r="P76" s="0">
+        <v>1</v>
       </c>
       <c r="Q76" s="0" t="s">
         <v>25</v>
@@ -6167,7 +6167,7 @@
         <v>46196.6612962963</v>
       </c>
       <c r="F77" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G77" s="0" t="s">
         <v>45</v>
@@ -6235,7 +6235,7 @@
         <v>46203.386967592596</v>
       </c>
       <c r="F78" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G78" s="0" t="s">
         <v>24</v>
@@ -6303,7 +6303,7 @@
         <v>46203.73695601852</v>
       </c>
       <c r="F79" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G79" s="0" t="s">
         <v>28</v>
@@ -6371,7 +6371,7 @@
         <v>46202.30238425926</v>
       </c>
       <c r="F80" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G80" s="0" t="s">
         <v>28</v>
@@ -6386,7 +6386,7 @@
         <v>28</v>
       </c>
       <c r="K80" s="0" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="L80" s="0" t="s">
         <v>25</v>
@@ -6406,8 +6406,8 @@
       <c r="Q80" s="0">
         <v>1</v>
       </c>
-      <c r="R80" s="0" t="s">
-        <v>25</v>
+      <c r="R80" s="0">
+        <v>0</v>
       </c>
       <c r="S80" s="0" t="s">
         <v>25</v>
@@ -6439,7 +6439,7 @@
         <v>46208.76116898148</v>
       </c>
       <c r="F81" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G81" s="0" t="s">
         <v>45</v>
@@ -6507,7 +6507,7 @@
         <v>46198.007743055554</v>
       </c>
       <c r="F82" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G82" s="0" t="s">
         <v>24</v>
@@ -6575,7 +6575,7 @@
         <v>46204.82892361111</v>
       </c>
       <c r="F83" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G83" s="0" t="s">
         <v>24</v>
@@ -6587,7 +6587,7 @@
         <v>24</v>
       </c>
       <c r="J83" s="0" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="K83" s="0" t="s">
         <v>25</v>
@@ -6607,8 +6607,8 @@
       <c r="P83" s="0">
         <v>1</v>
       </c>
-      <c r="Q83" s="0" t="s">
-        <v>25</v>
+      <c r="Q83" s="0">
+        <v>0</v>
       </c>
       <c r="R83" s="0" t="s">
         <v>25</v>
@@ -6643,7 +6643,7 @@
         <v>46211.026354166665</v>
       </c>
       <c r="F84" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G84" s="0" t="s">
         <v>24</v>
@@ -6673,7 +6673,7 @@
         <v>1</v>
       </c>
       <c r="P84" s="0">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q84" s="0" t="s">
         <v>25</v>
@@ -6711,7 +6711,7 @@
         <v>46206.49621527778</v>
       </c>
       <c r="F85" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G85" s="0" t="s">
         <v>28</v>
@@ -6723,7 +6723,7 @@
         <v>28</v>
       </c>
       <c r="J85" s="0" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="K85" s="0" t="s">
         <v>25</v>
@@ -6743,8 +6743,8 @@
       <c r="P85" s="0">
         <v>1</v>
       </c>
-      <c r="Q85" s="0" t="s">
-        <v>25</v>
+      <c r="Q85" s="0">
+        <v>0</v>
       </c>
       <c r="R85" s="0" t="s">
         <v>25</v>
@@ -6779,7 +6779,7 @@
         <v>46194.10880787037</v>
       </c>
       <c r="F86" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G86" s="0" t="s">
         <v>24</v>
@@ -6847,7 +6847,7 @@
         <v>46202.80762731482</v>
       </c>
       <c r="F87" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G87" s="0" t="s">
         <v>28</v>
@@ -6915,7 +6915,7 @@
         <v>46212.191030092596</v>
       </c>
       <c r="F88" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G88" s="0" t="s">
         <v>28</v>
@@ -6924,7 +6924,7 @@
         <v>28</v>
       </c>
       <c r="I88" s="0" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="J88" s="0" t="s">
         <v>25</v>
@@ -6944,8 +6944,8 @@
       <c r="O88" s="0">
         <v>1</v>
       </c>
-      <c r="P88" s="0" t="s">
-        <v>25</v>
+      <c r="P88" s="0">
+        <v>0</v>
       </c>
       <c r="Q88" s="0" t="s">
         <v>25</v>
@@ -6983,7 +6983,7 @@
         <v>46214.51880787037</v>
       </c>
       <c r="F89" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G89" s="0" t="s">
         <v>28</v>
@@ -7051,7 +7051,7 @@
         <v>46198.053506944445</v>
       </c>
       <c r="F90" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G90" s="0" t="s">
         <v>28</v>
@@ -7119,7 +7119,7 @@
         <v>46208.01679398148</v>
       </c>
       <c r="F91" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G91" s="0" t="s">
         <v>28</v>
@@ -7187,7 +7187,7 @@
         <v>46199.4216087963</v>
       </c>
       <c r="F92" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G92" s="0" t="s">
         <v>45</v>
@@ -7255,7 +7255,7 @@
         <v>46203.398622685185</v>
       </c>
       <c r="F93" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G93" s="0" t="s">
         <v>24</v>
@@ -7267,7 +7267,7 @@
         <v>24</v>
       </c>
       <c r="J93" s="0" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="K93" s="0" t="s">
         <v>25</v>
@@ -7287,8 +7287,8 @@
       <c r="P93" s="0">
         <v>1</v>
       </c>
-      <c r="Q93" s="0" t="s">
-        <v>25</v>
+      <c r="Q93" s="0">
+        <v>0</v>
       </c>
       <c r="R93" s="0" t="s">
         <v>25</v>
@@ -7323,7 +7323,7 @@
         <v>46204.071388888886</v>
       </c>
       <c r="F94" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G94" s="0" t="s">
         <v>24</v>
@@ -7391,7 +7391,7 @@
         <v>46204.81548611111</v>
       </c>
       <c r="F95" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G95" s="0" t="s">
         <v>24</v>
@@ -7400,7 +7400,7 @@
         <v>24</v>
       </c>
       <c r="I95" s="0" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="J95" s="0" t="s">
         <v>25</v>
@@ -7420,8 +7420,8 @@
       <c r="O95" s="0">
         <v>0</v>
       </c>
-      <c r="P95" s="0" t="s">
-        <v>25</v>
+      <c r="P95" s="0">
+        <v>1</v>
       </c>
       <c r="Q95" s="0" t="s">
         <v>25</v>
@@ -7459,7 +7459,7 @@
         <v>46207.340208333335</v>
       </c>
       <c r="F96" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G96" s="0" t="s">
         <v>28</v>
@@ -7471,7 +7471,7 @@
         <v>28</v>
       </c>
       <c r="J96" s="0" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="K96" s="0" t="s">
         <v>25</v>
@@ -7491,8 +7491,8 @@
       <c r="P96" s="0">
         <v>1</v>
       </c>
-      <c r="Q96" s="0" t="s">
-        <v>25</v>
+      <c r="Q96" s="0">
+        <v>0</v>
       </c>
       <c r="R96" s="0" t="s">
         <v>25</v>
@@ -7527,7 +7527,7 @@
         <v>46203.22761574074</v>
       </c>
       <c r="F97" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G97" s="0" t="s">
         <v>28</v>
@@ -7539,7 +7539,7 @@
         <v>28</v>
       </c>
       <c r="J97" s="0" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="K97" s="0" t="s">
         <v>25</v>
@@ -7559,8 +7559,8 @@
       <c r="P97" s="0">
         <v>0</v>
       </c>
-      <c r="Q97" s="0" t="s">
-        <v>25</v>
+      <c r="Q97" s="0">
+        <v>0</v>
       </c>
       <c r="R97" s="0" t="s">
         <v>25</v>
@@ -7595,7 +7595,7 @@
         <v>46203.73695601852</v>
       </c>
       <c r="F98" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G98" s="0" t="s">
         <v>28</v>
@@ -7663,7 +7663,7 @@
         <v>46209.27856481481</v>
       </c>
       <c r="F99" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G99" s="0" t="s">
         <v>28</v>
@@ -7731,7 +7731,7 @@
         <v>46203.241944444446</v>
       </c>
       <c r="F100" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G100" s="0" t="s">
         <v>28</v>
@@ -7799,7 +7799,7 @@
         <v>46200.90429398148</v>
       </c>
       <c r="F101" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G101" s="0" t="s">
         <v>24</v>
@@ -7829,7 +7829,7 @@
         <v>1</v>
       </c>
       <c r="P101" s="0">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q101" s="0" t="s">
         <v>25</v>
@@ -7867,7 +7867,7 @@
         <v>46201.17297453704</v>
       </c>
       <c r="F102" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G102" s="0" t="s">
         <v>28</v>
@@ -7935,7 +7935,7 @@
         <v>46197.398356481484</v>
       </c>
       <c r="F103" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G103" s="0" t="s">
         <v>24</v>
@@ -8003,7 +8003,7 @@
         <v>46198.06826388889</v>
       </c>
       <c r="F104" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G104" s="0" t="s">
         <v>24</v>
@@ -8015,7 +8015,7 @@
         <v>24</v>
       </c>
       <c r="J104" s="0" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="K104" s="0" t="s">
         <v>25</v>
@@ -8035,8 +8035,8 @@
       <c r="P104" s="0">
         <v>1</v>
       </c>
-      <c r="Q104" s="0" t="s">
-        <v>25</v>
+      <c r="Q104" s="0">
+        <v>0</v>
       </c>
       <c r="R104" s="0" t="s">
         <v>25</v>
@@ -8071,7 +8071,7 @@
         <v>46204.81618055556</v>
       </c>
       <c r="F105" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G105" s="0" t="s">
         <v>24</v>
@@ -8080,7 +8080,7 @@
         <v>24</v>
       </c>
       <c r="I105" s="0" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="J105" s="0" t="s">
         <v>25</v>
@@ -8100,8 +8100,8 @@
       <c r="O105" s="0">
         <v>0</v>
       </c>
-      <c r="P105" s="0" t="s">
-        <v>25</v>
+      <c r="P105" s="0">
+        <v>1</v>
       </c>
       <c r="Q105" s="0" t="s">
         <v>25</v>
@@ -8139,7 +8139,7 @@
         <v>46184.345671296294</v>
       </c>
       <c r="F106" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G106" s="0" t="s">
         <v>24</v>
@@ -8148,7 +8148,7 @@
         <v>24</v>
       </c>
       <c r="I106" s="0" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="J106" s="0" t="s">
         <v>25</v>
@@ -8168,8 +8168,8 @@
       <c r="O106" s="0">
         <v>1</v>
       </c>
-      <c r="P106" s="0" t="s">
-        <v>25</v>
+      <c r="P106" s="0">
+        <v>0</v>
       </c>
       <c r="Q106" s="0" t="s">
         <v>25</v>
@@ -8207,7 +8207,7 @@
         <v>46198.76695601852</v>
       </c>
       <c r="F107" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G107" s="0" t="s">
         <v>24</v>
@@ -8219,7 +8219,7 @@
         <v>24</v>
       </c>
       <c r="J107" s="0" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="K107" s="0" t="s">
         <v>25</v>
@@ -8239,8 +8239,8 @@
       <c r="P107" s="0">
         <v>1</v>
       </c>
-      <c r="Q107" s="0" t="s">
-        <v>25</v>
+      <c r="Q107" s="0">
+        <v>0</v>
       </c>
       <c r="R107" s="0" t="s">
         <v>25</v>
@@ -8275,7 +8275,7 @@
         <v>46199.06940972222</v>
       </c>
       <c r="F108" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G108" s="0" t="s">
         <v>45</v>
@@ -8287,7 +8287,7 @@
         <v>45</v>
       </c>
       <c r="J108" s="0" t="s">
-        <v>25</v>
+        <v>45</v>
       </c>
       <c r="K108" s="0" t="s">
         <v>25</v>
@@ -8307,8 +8307,8 @@
       <c r="P108" s="0">
         <v>1</v>
       </c>
-      <c r="Q108" s="0" t="s">
-        <v>25</v>
+      <c r="Q108" s="0">
+        <v>0</v>
       </c>
       <c r="R108" s="0" t="s">
         <v>25</v>
@@ -8343,7 +8343,7 @@
         <v>46207.38381944445</v>
       </c>
       <c r="F109" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G109" s="0" t="s">
         <v>28</v>
@@ -8355,7 +8355,7 @@
         <v>28</v>
       </c>
       <c r="J109" s="0" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="K109" s="0" t="s">
         <v>25</v>
@@ -8375,8 +8375,8 @@
       <c r="P109" s="0">
         <v>1</v>
       </c>
-      <c r="Q109" s="0" t="s">
-        <v>25</v>
+      <c r="Q109" s="0">
+        <v>0</v>
       </c>
       <c r="R109" s="0" t="s">
         <v>25</v>
@@ -8411,7 +8411,7 @@
         <v>46198.764710648145</v>
       </c>
       <c r="F110" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G110" s="0" t="s">
         <v>24</v>
@@ -8423,7 +8423,7 @@
         <v>24</v>
       </c>
       <c r="J110" s="0" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="K110" s="0" t="s">
         <v>25</v>
@@ -8443,8 +8443,8 @@
       <c r="P110" s="0">
         <v>1</v>
       </c>
-      <c r="Q110" s="0" t="s">
-        <v>25</v>
+      <c r="Q110" s="0">
+        <v>0</v>
       </c>
       <c r="R110" s="0" t="s">
         <v>25</v>
@@ -8479,7 +8479,7 @@
         <v>46208.60445601852</v>
       </c>
       <c r="F111" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G111" s="0" t="s">
         <v>28</v>
@@ -8547,7 +8547,7 @@
         <v>46198.06826388889</v>
       </c>
       <c r="F112" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G112" s="0" t="s">
         <v>45</v>
@@ -8559,7 +8559,7 @@
         <v>45</v>
       </c>
       <c r="J112" s="0" t="s">
-        <v>25</v>
+        <v>45</v>
       </c>
       <c r="K112" s="0" t="s">
         <v>25</v>
@@ -8579,8 +8579,8 @@
       <c r="P112" s="0">
         <v>1</v>
       </c>
-      <c r="Q112" s="0" t="s">
-        <v>25</v>
+      <c r="Q112" s="0">
+        <v>0</v>
       </c>
       <c r="R112" s="0" t="s">
         <v>25</v>
@@ -8615,7 +8615,7 @@
         <v>46198.7566087963</v>
       </c>
       <c r="F113" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G113" s="0" t="s">
         <v>24</v>
@@ -8627,7 +8627,7 @@
         <v>24</v>
       </c>
       <c r="J113" s="0" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="K113" s="0" t="s">
         <v>25</v>
@@ -8647,8 +8647,8 @@
       <c r="P113" s="0">
         <v>1</v>
       </c>
-      <c r="Q113" s="0" t="s">
-        <v>25</v>
+      <c r="Q113" s="0">
+        <v>0</v>
       </c>
       <c r="R113" s="0" t="s">
         <v>25</v>
@@ -8683,7 +8683,7 @@
         <v>46204.591203703705</v>
       </c>
       <c r="F114" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G114" s="0" t="s">
         <v>28</v>
@@ -8692,7 +8692,7 @@
         <v>28</v>
       </c>
       <c r="I114" s="0" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="J114" s="0" t="s">
         <v>25</v>
@@ -8712,8 +8712,8 @@
       <c r="O114" s="0">
         <v>0</v>
       </c>
-      <c r="P114" s="0" t="s">
-        <v>25</v>
+      <c r="P114" s="0">
+        <v>0</v>
       </c>
       <c r="Q114" s="0" t="s">
         <v>25</v>
@@ -8751,7 +8751,7 @@
         <v>46203.38690972222</v>
       </c>
       <c r="F115" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G115" s="0" t="s">
         <v>24</v>
@@ -8819,7 +8819,7 @@
         <v>46199.954201388886</v>
       </c>
       <c r="F116" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G116" s="0" t="s">
         <v>28</v>
@@ -8852,7 +8852,7 @@
         <v>1</v>
       </c>
       <c r="Q116" s="0">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R116" s="0" t="s">
         <v>25</v>
@@ -8887,7 +8887,7 @@
         <v>46199.06940972222</v>
       </c>
       <c r="F117" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G117" s="0" t="s">
         <v>45</v>
@@ -8899,7 +8899,7 @@
         <v>45</v>
       </c>
       <c r="J117" s="0" t="s">
-        <v>25</v>
+        <v>45</v>
       </c>
       <c r="K117" s="0" t="s">
         <v>25</v>
@@ -8919,8 +8919,8 @@
       <c r="P117" s="0">
         <v>1</v>
       </c>
-      <c r="Q117" s="0" t="s">
-        <v>25</v>
+      <c r="Q117" s="0">
+        <v>0</v>
       </c>
       <c r="R117" s="0" t="s">
         <v>25</v>
@@ -8955,7 +8955,7 @@
         <v>46193.45674768519</v>
       </c>
       <c r="F118" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G118" s="0" t="s">
         <v>24</v>
@@ -9023,7 +9023,7 @@
         <v>46211.339479166665</v>
       </c>
       <c r="F119" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G119" s="0" t="s">
         <v>24</v>
@@ -9091,7 +9091,7 @@
         <v>46184.344409722224</v>
       </c>
       <c r="F120" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G120" s="0" t="s">
         <v>24</v>
@@ -9100,7 +9100,7 @@
         <v>24</v>
       </c>
       <c r="I120" s="0" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="J120" s="0" t="s">
         <v>25</v>
@@ -9120,8 +9120,8 @@
       <c r="O120" s="0">
         <v>1</v>
       </c>
-      <c r="P120" s="0" t="s">
-        <v>25</v>
+      <c r="P120" s="0">
+        <v>0</v>
       </c>
       <c r="Q120" s="0" t="s">
         <v>25</v>
@@ -9159,7 +9159,7 @@
         <v>46196.43208333333</v>
       </c>
       <c r="F121" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G121" s="0" t="s">
         <v>28</v>
@@ -9227,7 +9227,7 @@
         <v>46204.591203703705</v>
       </c>
       <c r="F122" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G122" s="0" t="s">
         <v>28</v>
@@ -9236,7 +9236,7 @@
         <v>28</v>
       </c>
       <c r="I122" s="0" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="J122" s="0" t="s">
         <v>25</v>
@@ -9256,8 +9256,8 @@
       <c r="O122" s="0">
         <v>0</v>
       </c>
-      <c r="P122" s="0" t="s">
-        <v>25</v>
+      <c r="P122" s="0">
+        <v>0</v>
       </c>
       <c r="Q122" s="0" t="s">
         <v>25</v>
@@ -9295,7 +9295,7 @@
         <v>46212.38707175926</v>
       </c>
       <c r="F123" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G123" s="0" t="s">
         <v>28</v>
@@ -9363,7 +9363,7 @@
         <v>46205.85377314815</v>
       </c>
       <c r="F124" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G124" s="0" t="s">
         <v>24</v>
@@ -9375,7 +9375,7 @@
         <v>24</v>
       </c>
       <c r="J124" s="0" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="K124" s="0" t="s">
         <v>25</v>
@@ -9395,8 +9395,8 @@
       <c r="P124" s="0">
         <v>1</v>
       </c>
-      <c r="Q124" s="0" t="s">
-        <v>25</v>
+      <c r="Q124" s="0">
+        <v>0</v>
       </c>
       <c r="R124" s="0" t="s">
         <v>25</v>
@@ -9431,7 +9431,7 @@
         <v>46204.81548611111</v>
       </c>
       <c r="F125" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G125" s="0" t="s">
         <v>24</v>
@@ -9440,7 +9440,7 @@
         <v>24</v>
       </c>
       <c r="I125" s="0" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="J125" s="0" t="s">
         <v>25</v>
@@ -9460,8 +9460,8 @@
       <c r="O125" s="0">
         <v>0</v>
       </c>
-      <c r="P125" s="0" t="s">
-        <v>25</v>
+      <c r="P125" s="0">
+        <v>1</v>
       </c>
       <c r="Q125" s="0" t="s">
         <v>25</v>
@@ -9499,7 +9499,7 @@
         <v>46194.496782407405</v>
       </c>
       <c r="F126" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G126" s="0" t="s">
         <v>45</v>
@@ -9535,7 +9535,7 @@
         <v>1</v>
       </c>
       <c r="R126" s="0">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S126" s="0" t="s">
         <v>25</v>
@@ -9567,7 +9567,7 @@
         <v>46206.041817129626</v>
       </c>
       <c r="F127" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G127" s="0" t="s">
         <v>28</v>
@@ -9635,7 +9635,7 @@
         <v>46211.74564814815</v>
       </c>
       <c r="F128" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G128" s="0" t="s">
         <v>24</v>
@@ -9644,7 +9644,7 @@
         <v>24</v>
       </c>
       <c r="I128" s="0" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="J128" s="0" t="s">
         <v>25</v>
@@ -9664,8 +9664,8 @@
       <c r="O128" s="0">
         <v>0</v>
       </c>
-      <c r="P128" s="0" t="s">
-        <v>25</v>
+      <c r="P128" s="0">
+        <v>1</v>
       </c>
       <c r="Q128" s="0" t="s">
         <v>25</v>
@@ -9703,7 +9703,7 @@
         <v>46198.76357638889</v>
       </c>
       <c r="F129" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G129" s="0" t="s">
         <v>24</v>
@@ -9715,7 +9715,7 @@
         <v>24</v>
       </c>
       <c r="J129" s="0" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="K129" s="0" t="s">
         <v>25</v>
@@ -9735,8 +9735,8 @@
       <c r="P129" s="0">
         <v>1</v>
       </c>
-      <c r="Q129" s="0" t="s">
-        <v>25</v>
+      <c r="Q129" s="0">
+        <v>0</v>
       </c>
       <c r="R129" s="0" t="s">
         <v>25</v>
@@ -9771,7 +9771,7 @@
         <v>46214.41127314815</v>
       </c>
       <c r="F130" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G130" s="0" t="s">
         <v>28</v>
@@ -9839,7 +9839,7 @@
         <v>46210.39944444445</v>
       </c>
       <c r="F131" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G131" s="0" t="s">
         <v>24</v>
@@ -9907,7 +9907,7 @@
         <v>46203.900046296294</v>
       </c>
       <c r="F132" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G132" s="0" t="s">
         <v>45</v>
@@ -9919,7 +9919,7 @@
         <v>45</v>
       </c>
       <c r="J132" s="0" t="s">
-        <v>25</v>
+        <v>45</v>
       </c>
       <c r="K132" s="0" t="s">
         <v>25</v>
@@ -9939,8 +9939,8 @@
       <c r="P132" s="0">
         <v>1</v>
       </c>
-      <c r="Q132" s="0" t="s">
-        <v>25</v>
+      <c r="Q132" s="0">
+        <v>0</v>
       </c>
       <c r="R132" s="0" t="s">
         <v>25</v>
@@ -9975,7 +9975,7 @@
         <v>46198.75818287037</v>
       </c>
       <c r="F133" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G133" s="0" t="s">
         <v>24</v>
@@ -9987,7 +9987,7 @@
         <v>24</v>
       </c>
       <c r="J133" s="0" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="K133" s="0" t="s">
         <v>25</v>
@@ -10007,8 +10007,8 @@
       <c r="P133" s="0">
         <v>1</v>
       </c>
-      <c r="Q133" s="0" t="s">
-        <v>25</v>
+      <c r="Q133" s="0">
+        <v>0</v>
       </c>
       <c r="R133" s="0" t="s">
         <v>25</v>
@@ -10043,7 +10043,7 @@
         <v>46199.24039351852</v>
       </c>
       <c r="F134" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G134" s="0" t="s">
         <v>28</v>
@@ -10111,7 +10111,7 @@
         <v>46207.7878125</v>
       </c>
       <c r="F135" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G135" s="0" t="s">
         <v>28</v>
@@ -10179,7 +10179,7 @@
         <v>46200.88856481481</v>
       </c>
       <c r="F136" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G136" s="0" t="s">
         <v>45</v>
@@ -10247,7 +10247,7 @@
         <v>46207.091145833336</v>
       </c>
       <c r="F137" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G137" s="0" t="s">
         <v>28</v>
@@ -10259,7 +10259,7 @@
         <v>28</v>
       </c>
       <c r="J137" s="0" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="K137" s="0" t="s">
         <v>25</v>
@@ -10279,8 +10279,8 @@
       <c r="P137" s="0">
         <v>1</v>
       </c>
-      <c r="Q137" s="0" t="s">
-        <v>25</v>
+      <c r="Q137" s="0">
+        <v>0</v>
       </c>
       <c r="R137" s="0" t="s">
         <v>25</v>
@@ -10315,7 +10315,7 @@
         <v>46209.81253472222</v>
       </c>
       <c r="F138" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G138" s="0" t="s">
         <v>24</v>
@@ -10383,7 +10383,7 @@
         <v>46204.81548611111</v>
       </c>
       <c r="F139" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G139" s="0" t="s">
         <v>24</v>
@@ -10392,7 +10392,7 @@
         <v>24</v>
       </c>
       <c r="I139" s="0" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="J139" s="0" t="s">
         <v>25</v>
@@ -10412,8 +10412,8 @@
       <c r="O139" s="0">
         <v>0</v>
       </c>
-      <c r="P139" s="0" t="s">
-        <v>25</v>
+      <c r="P139" s="0">
+        <v>1</v>
       </c>
       <c r="Q139" s="0" t="s">
         <v>25</v>
@@ -10451,7 +10451,7 @@
         <v>46208.76133101852</v>
       </c>
       <c r="F140" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G140" s="0" t="s">
         <v>24</v>
@@ -10519,7 +10519,7 @@
         <v>46210.11184027778</v>
       </c>
       <c r="F141" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G141" s="0" t="s">
         <v>24</v>
@@ -10528,7 +10528,7 @@
         <v>24</v>
       </c>
       <c r="I141" s="0" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="J141" s="0" t="s">
         <v>25</v>
@@ -10548,8 +10548,8 @@
       <c r="O141" s="0">
         <v>1</v>
       </c>
-      <c r="P141" s="0" t="s">
-        <v>25</v>
+      <c r="P141" s="0">
+        <v>0</v>
       </c>
       <c r="Q141" s="0" t="s">
         <v>25</v>
@@ -10587,7 +10587,7 @@
         <v>46202.603946759256</v>
       </c>
       <c r="F142" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G142" s="0" t="s">
         <v>24</v>
@@ -10655,7 +10655,7 @@
         <v>46208.28020833333</v>
       </c>
       <c r="F143" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G143" s="0" t="s">
         <v>45</v>
@@ -10723,7 +10723,7 @@
         <v>46203.665925925925</v>
       </c>
       <c r="F144" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G144" s="0" t="s">
         <v>24</v>
@@ -10735,7 +10735,7 @@
         <v>24</v>
       </c>
       <c r="J144" s="0" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="K144" s="0" t="s">
         <v>25</v>
@@ -10755,8 +10755,8 @@
       <c r="P144" s="0">
         <v>1</v>
       </c>
-      <c r="Q144" s="0" t="s">
-        <v>25</v>
+      <c r="Q144" s="0">
+        <v>0</v>
       </c>
       <c r="R144" s="0" t="s">
         <v>25</v>
@@ -10791,7 +10791,7 @@
         <v>46187.9200462963</v>
       </c>
       <c r="F145" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G145" s="0" t="s">
         <v>24</v>
@@ -10859,7 +10859,7 @@
         <v>46204.36974537037</v>
       </c>
       <c r="F146" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G146" s="0" t="s">
         <v>28</v>
@@ -10927,7 +10927,7 @@
         <v>46201.332870370374</v>
       </c>
       <c r="F147" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G147" s="0" t="s">
         <v>24</v>
@@ -10995,7 +10995,7 @@
         <v>46197.03113425926</v>
       </c>
       <c r="F148" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G148" s="0" t="s">
         <v>24</v>
@@ -11063,7 +11063,7 @@
         <v>46212.285219907404</v>
       </c>
       <c r="F149" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G149" s="0" t="s">
         <v>28</v>
@@ -11131,7 +11131,7 @@
         <v>46200.98619212963</v>
       </c>
       <c r="F150" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G150" s="0" t="s">
         <v>28</v>
@@ -11146,7 +11146,7 @@
         <v>28</v>
       </c>
       <c r="K150" s="0" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="L150" s="0" t="s">
         <v>25</v>
@@ -11166,8 +11166,8 @@
       <c r="Q150" s="0">
         <v>0</v>
       </c>
-      <c r="R150" s="0" t="s">
-        <v>25</v>
+      <c r="R150" s="0">
+        <v>0</v>
       </c>
       <c r="S150" s="0" t="s">
         <v>25</v>
@@ -11199,7 +11199,7 @@
         <v>46212.06758101852</v>
       </c>
       <c r="F151" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G151" s="0" t="s">
         <v>28</v>
@@ -11208,7 +11208,7 @@
         <v>28</v>
       </c>
       <c r="I151" s="0" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="J151" s="0" t="s">
         <v>25</v>
@@ -11228,8 +11228,8 @@
       <c r="O151" s="0">
         <v>0</v>
       </c>
-      <c r="P151" s="0" t="s">
-        <v>25</v>
+      <c r="P151" s="0">
+        <v>0</v>
       </c>
       <c r="Q151" s="0" t="s">
         <v>25</v>
@@ -11267,7 +11267,7 @@
         <v>46207.18613425926</v>
       </c>
       <c r="F152" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G152" s="0" t="s">
         <v>28</v>
@@ -11335,7 +11335,7 @@
         <v>46210.8569212963</v>
       </c>
       <c r="F153" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G153" s="0" t="s">
         <v>28</v>
@@ -11365,7 +11365,7 @@
         <v>1</v>
       </c>
       <c r="P153" s="0">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q153" s="0" t="s">
         <v>25</v>
@@ -11403,7 +11403,7 @@
         <v>46198.763344907406</v>
       </c>
       <c r="F154" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G154" s="0" t="s">
         <v>24</v>
@@ -11415,7 +11415,7 @@
         <v>24</v>
       </c>
       <c r="J154" s="0" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="K154" s="0" t="s">
         <v>25</v>
@@ -11435,8 +11435,8 @@
       <c r="P154" s="0">
         <v>1</v>
       </c>
-      <c r="Q154" s="0" t="s">
-        <v>25</v>
+      <c r="Q154" s="0">
+        <v>0</v>
       </c>
       <c r="R154" s="0" t="s">
         <v>25</v>
@@ -11471,7 +11471,7 @@
         <v>46204.815416666665</v>
       </c>
       <c r="F155" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G155" s="0" t="s">
         <v>24</v>
@@ -11480,7 +11480,7 @@
         <v>24</v>
       </c>
       <c r="I155" s="0" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="J155" s="0" t="s">
         <v>25</v>
@@ -11500,8 +11500,8 @@
       <c r="O155" s="0">
         <v>0</v>
       </c>
-      <c r="P155" s="0" t="s">
-        <v>25</v>
+      <c r="P155" s="0">
+        <v>1</v>
       </c>
       <c r="Q155" s="0" t="s">
         <v>25</v>
@@ -11539,7 +11539,7 @@
         <v>46198.86886574074</v>
       </c>
       <c r="F156" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G156" s="0" t="s">
         <v>28</v>
@@ -11607,7 +11607,7 @@
         <v>46198.76422453704</v>
       </c>
       <c r="F157" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G157" s="0" t="s">
         <v>24</v>
@@ -11619,7 +11619,7 @@
         <v>24</v>
       </c>
       <c r="J157" s="0" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="K157" s="0" t="s">
         <v>25</v>
@@ -11639,8 +11639,8 @@
       <c r="P157" s="0">
         <v>1</v>
       </c>
-      <c r="Q157" s="0" t="s">
-        <v>25</v>
+      <c r="Q157" s="0">
+        <v>0</v>
       </c>
       <c r="R157" s="0" t="s">
         <v>25</v>
@@ -11675,7 +11675,7 @@
         <v>46206.29314814815</v>
       </c>
       <c r="F158" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G158" s="0" t="s">
         <v>45</v>
@@ -11705,7 +11705,7 @@
         <v>1</v>
       </c>
       <c r="P158" s="0">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q158" s="0" t="s">
         <v>25</v>
@@ -11743,7 +11743,7 @@
         <v>46206.39832175926</v>
       </c>
       <c r="F159" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G159" s="0" t="s">
         <v>28</v>
@@ -11755,7 +11755,7 @@
         <v>28</v>
       </c>
       <c r="J159" s="0" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="K159" s="0" t="s">
         <v>25</v>
@@ -11775,8 +11775,8 @@
       <c r="P159" s="0">
         <v>0</v>
       </c>
-      <c r="Q159" s="0" t="s">
-        <v>25</v>
+      <c r="Q159" s="0">
+        <v>0</v>
       </c>
       <c r="R159" s="0" t="s">
         <v>25</v>
@@ -11811,7 +11811,7 @@
         <v>46201.828206018516</v>
       </c>
       <c r="F160" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G160" s="0" t="s">
         <v>28</v>
@@ -11826,7 +11826,7 @@
         <v>28</v>
       </c>
       <c r="K160" s="0" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="L160" s="0" t="s">
         <v>25</v>
@@ -11846,8 +11846,8 @@
       <c r="Q160" s="0">
         <v>1</v>
       </c>
-      <c r="R160" s="0" t="s">
-        <v>25</v>
+      <c r="R160" s="0">
+        <v>0</v>
       </c>
       <c r="S160" s="0" t="s">
         <v>25</v>
@@ -11879,7 +11879,7 @@
         <v>46198.13486111111</v>
       </c>
       <c r="F161" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G161" s="0" t="s">
         <v>24</v>
@@ -11947,7 +11947,7 @@
         <v>46184.34568287037</v>
       </c>
       <c r="F162" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G162" s="0" t="s">
         <v>24</v>
@@ -11956,7 +11956,7 @@
         <v>24</v>
       </c>
       <c r="I162" s="0" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="J162" s="0" t="s">
         <v>25</v>
@@ -11976,8 +11976,8 @@
       <c r="O162" s="0">
         <v>1</v>
       </c>
-      <c r="P162" s="0" t="s">
-        <v>25</v>
+      <c r="P162" s="0">
+        <v>0</v>
       </c>
       <c r="Q162" s="0" t="s">
         <v>25</v>
@@ -12015,7 +12015,7 @@
         <v>46198.487546296295</v>
       </c>
       <c r="F163" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G163" s="0" t="s">
         <v>28</v>
@@ -12083,7 +12083,7 @@
         <v>46204.815405092595</v>
       </c>
       <c r="F164" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G164" s="0" t="s">
         <v>24</v>
@@ -12092,7 +12092,7 @@
         <v>24</v>
       </c>
       <c r="I164" s="0" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="J164" s="0" t="s">
         <v>25</v>
@@ -12112,8 +12112,8 @@
       <c r="O164" s="0">
         <v>0</v>
       </c>
-      <c r="P164" s="0" t="s">
-        <v>25</v>
+      <c r="P164" s="0">
+        <v>1</v>
       </c>
       <c r="Q164" s="0" t="s">
         <v>25</v>
@@ -12151,7 +12151,7 @@
         <v>46204.815405092595</v>
       </c>
       <c r="F165" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G165" s="0" t="s">
         <v>24</v>
@@ -12160,7 +12160,7 @@
         <v>24</v>
       </c>
       <c r="I165" s="0" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="J165" s="0" t="s">
         <v>25</v>
@@ -12180,8 +12180,8 @@
       <c r="O165" s="0">
         <v>0</v>
       </c>
-      <c r="P165" s="0" t="s">
-        <v>25</v>
+      <c r="P165" s="0">
+        <v>1</v>
       </c>
       <c r="Q165" s="0" t="s">
         <v>25</v>
@@ -12219,7 +12219,7 @@
         <v>46199.37</v>
       </c>
       <c r="F166" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G166" s="0" t="s">
         <v>28</v>
@@ -12287,7 +12287,7 @@
         <v>46200.507418981484</v>
       </c>
       <c r="F167" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G167" s="0" t="s">
         <v>28</v>
@@ -12323,7 +12323,7 @@
         <v>1</v>
       </c>
       <c r="R167" s="0">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S167" s="0" t="s">
         <v>25</v>
@@ -12355,7 +12355,7 @@
         <v>46208.7612037037</v>
       </c>
       <c r="F168" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G168" s="0" t="s">
         <v>45</v>
@@ -12385,7 +12385,7 @@
         <v>1</v>
       </c>
       <c r="P168" s="0">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q168" s="0" t="s">
         <v>25</v>
@@ -12423,7 +12423,7 @@
         <v>46204.81548611111</v>
       </c>
       <c r="F169" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G169" s="0" t="s">
         <v>24</v>
@@ -12432,7 +12432,7 @@
         <v>24</v>
       </c>
       <c r="I169" s="0" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="J169" s="0" t="s">
         <v>25</v>
@@ -12452,8 +12452,8 @@
       <c r="O169" s="0">
         <v>0</v>
       </c>
-      <c r="P169" s="0" t="s">
-        <v>25</v>
+      <c r="P169" s="0">
+        <v>1</v>
       </c>
       <c r="Q169" s="0" t="s">
         <v>25</v>
@@ -12491,7 +12491,7 @@
         <v>46206.616875</v>
       </c>
       <c r="F170" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G170" s="0" t="s">
         <v>28</v>
@@ -12559,7 +12559,7 @@
         <v>46206.85376157407</v>
       </c>
       <c r="F171" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G171" s="0" t="s">
         <v>24</v>
@@ -12627,7 +12627,7 @@
         <v>46204.815416666665</v>
       </c>
       <c r="F172" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G172" s="0" t="s">
         <v>24</v>
@@ -12636,7 +12636,7 @@
         <v>24</v>
       </c>
       <c r="I172" s="0" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="J172" s="0" t="s">
         <v>25</v>
@@ -12656,8 +12656,8 @@
       <c r="O172" s="0">
         <v>0</v>
       </c>
-      <c r="P172" s="0" t="s">
-        <v>25</v>
+      <c r="P172" s="0">
+        <v>1</v>
       </c>
       <c r="Q172" s="0" t="s">
         <v>25</v>
@@ -12695,7 +12695,7 @@
         <v>46215.346342592595</v>
       </c>
       <c r="F173" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G173" s="0" t="s">
         <v>45</v>
@@ -12763,7 +12763,7 @@
         <v>46208.34142361111</v>
       </c>
       <c r="F174" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G174" s="0" t="s">
         <v>45</v>
@@ -12831,7 +12831,7 @@
         <v>46184.34611111111</v>
       </c>
       <c r="F175" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G175" s="0" t="s">
         <v>24</v>
@@ -12840,7 +12840,7 @@
         <v>24</v>
       </c>
       <c r="I175" s="0" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="J175" s="0" t="s">
         <v>25</v>
@@ -12860,8 +12860,8 @@
       <c r="O175" s="0">
         <v>1</v>
       </c>
-      <c r="P175" s="0" t="s">
-        <v>25</v>
+      <c r="P175" s="0">
+        <v>0</v>
       </c>
       <c r="Q175" s="0" t="s">
         <v>25</v>
@@ -12899,7 +12899,7 @@
         <v>46207.44116898148</v>
       </c>
       <c r="F176" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G176" s="0" t="s">
         <v>45</v>
@@ -12967,7 +12967,7 @@
         <v>46213.12200231481</v>
       </c>
       <c r="F177" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G177" s="0" t="s">
         <v>28</v>
@@ -13035,7 +13035,7 @@
         <v>46211.78650462963</v>
       </c>
       <c r="F178" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G178" s="0" t="s">
         <v>28</v>
@@ -13103,7 +13103,7 @@
         <v>46205.74003472222</v>
       </c>
       <c r="F179" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G179" s="0" t="s">
         <v>45</v>
@@ -13115,7 +13115,7 @@
         <v>45</v>
       </c>
       <c r="J179" s="0" t="s">
-        <v>25</v>
+        <v>45</v>
       </c>
       <c r="K179" s="0" t="s">
         <v>25</v>
@@ -13135,8 +13135,8 @@
       <c r="P179" s="0">
         <v>0</v>
       </c>
-      <c r="Q179" s="0" t="s">
-        <v>25</v>
+      <c r="Q179" s="0">
+        <v>0</v>
       </c>
       <c r="R179" s="0" t="s">
         <v>25</v>
@@ -13171,7 +13171,7 @@
         <v>46214.6358912037</v>
       </c>
       <c r="F180" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G180" s="0" t="s">
         <v>28</v>
@@ -13239,7 +13239,7 @@
         <v>46199.95371527778</v>
       </c>
       <c r="F181" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G181" s="0" t="s">
         <v>45</v>
@@ -13307,7 +13307,7 @@
         <v>46205.07099537037</v>
       </c>
       <c r="F182" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G182" s="0" t="s">
         <v>24</v>
@@ -13375,7 +13375,7 @@
         <v>46215.09512731482</v>
       </c>
       <c r="F183" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G183" s="0" t="s">
         <v>28</v>
@@ -13443,7 +13443,7 @@
         <v>46203.39921296296</v>
       </c>
       <c r="F184" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G184" s="0" t="s">
         <v>24</v>
@@ -13455,7 +13455,7 @@
         <v>24</v>
       </c>
       <c r="J184" s="0" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="K184" s="0" t="s">
         <v>25</v>
@@ -13475,8 +13475,8 @@
       <c r="P184" s="0">
         <v>1</v>
       </c>
-      <c r="Q184" s="0" t="s">
-        <v>25</v>
+      <c r="Q184" s="0">
+        <v>0</v>
       </c>
       <c r="R184" s="0" t="s">
         <v>25</v>
@@ -13511,7 +13511,7 @@
         <v>46206.91523148148</v>
       </c>
       <c r="F185" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G185" s="0" t="s">
         <v>24</v>
@@ -13541,7 +13541,7 @@
         <v>1</v>
       </c>
       <c r="P185" s="0">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q185" s="0" t="s">
         <v>25</v>
@@ -13579,7 +13579,7 @@
         <v>46199.06940972222</v>
       </c>
       <c r="F186" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G186" s="0" t="s">
         <v>24</v>
@@ -13591,7 +13591,7 @@
         <v>24</v>
       </c>
       <c r="J186" s="0" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="K186" s="0" t="s">
         <v>25</v>
@@ -13611,8 +13611,8 @@
       <c r="P186" s="0">
         <v>1</v>
       </c>
-      <c r="Q186" s="0" t="s">
-        <v>25</v>
+      <c r="Q186" s="0">
+        <v>0</v>
       </c>
       <c r="R186" s="0" t="s">
         <v>25</v>
@@ -13647,7 +13647,7 @@
         <v>46212.73332175926</v>
       </c>
       <c r="F187" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G187" s="0" t="s">
         <v>28</v>
@@ -13715,7 +13715,7 @@
         <v>46199.395949074074</v>
       </c>
       <c r="F188" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G188" s="0" t="s">
         <v>28</v>
@@ -13783,7 +13783,7 @@
         <v>46184.34570601852</v>
       </c>
       <c r="F189" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G189" s="0" t="s">
         <v>24</v>
@@ -13792,7 +13792,7 @@
         <v>24</v>
       </c>
       <c r="I189" s="0" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="J189" s="0" t="s">
         <v>25</v>
@@ -13812,8 +13812,8 @@
       <c r="O189" s="0">
         <v>1</v>
       </c>
-      <c r="P189" s="0" t="s">
-        <v>25</v>
+      <c r="P189" s="0">
+        <v>0</v>
       </c>
       <c r="Q189" s="0" t="s">
         <v>25</v>
@@ -13851,7 +13851,7 @@
         <v>46198.756527777776</v>
       </c>
       <c r="F190" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G190" s="0" t="s">
         <v>24</v>
@@ -13863,7 +13863,7 @@
         <v>24</v>
       </c>
       <c r="J190" s="0" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="K190" s="0" t="s">
         <v>25</v>
@@ -13883,8 +13883,8 @@
       <c r="P190" s="0">
         <v>1</v>
       </c>
-      <c r="Q190" s="0" t="s">
-        <v>25</v>
+      <c r="Q190" s="0">
+        <v>0</v>
       </c>
       <c r="R190" s="0" t="s">
         <v>25</v>
@@ -13919,7 +13919,7 @@
         <v>46208.76128472222</v>
       </c>
       <c r="F191" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G191" s="0" t="s">
         <v>24</v>
@@ -13987,7 +13987,7 @@
         <v>46198.76427083334</v>
       </c>
       <c r="F192" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G192" s="0" t="s">
         <v>24</v>
@@ -13999,7 +13999,7 @@
         <v>24</v>
       </c>
       <c r="J192" s="0" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="K192" s="0" t="s">
         <v>25</v>
@@ -14019,8 +14019,8 @@
       <c r="P192" s="0">
         <v>1</v>
       </c>
-      <c r="Q192" s="0" t="s">
-        <v>25</v>
+      <c r="Q192" s="0">
+        <v>0</v>
       </c>
       <c r="R192" s="0" t="s">
         <v>25</v>
@@ -14055,7 +14055,7 @@
         <v>46196.08101851852</v>
       </c>
       <c r="F193" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G193" s="0" t="s">
         <v>24</v>
@@ -14123,7 +14123,7 @@
         <v>46207.28523148148</v>
       </c>
       <c r="F194" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G194" s="0" t="s">
         <v>24</v>
@@ -14191,7 +14191,7 @@
         <v>46196.788564814815</v>
       </c>
       <c r="F195" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G195" s="0" t="s">
         <v>24</v>
@@ -14203,7 +14203,7 @@
         <v>24</v>
       </c>
       <c r="J195" s="0" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="K195" s="0" t="s">
         <v>25</v>
@@ -14223,8 +14223,8 @@
       <c r="P195" s="0">
         <v>1</v>
       </c>
-      <c r="Q195" s="0" t="s">
-        <v>25</v>
+      <c r="Q195" s="0">
+        <v>0</v>
       </c>
       <c r="R195" s="0" t="s">
         <v>25</v>
@@ -14259,7 +14259,7 @@
         <v>46200.45096064815</v>
       </c>
       <c r="F196" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G196" s="0" t="s">
         <v>45</v>
@@ -14327,7 +14327,7 @@
         <v>46213.44936342593</v>
       </c>
       <c r="F197" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G197" s="0" t="s">
         <v>28</v>
@@ -14395,7 +14395,7 @@
         <v>46207.18237268519</v>
       </c>
       <c r="F198" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G198" s="0" t="s">
         <v>24</v>
@@ -14407,7 +14407,7 @@
         <v>24</v>
       </c>
       <c r="J198" s="0" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="K198" s="0" t="s">
         <v>25</v>
@@ -14427,8 +14427,8 @@
       <c r="P198" s="0">
         <v>1</v>
       </c>
-      <c r="Q198" s="0" t="s">
-        <v>25</v>
+      <c r="Q198" s="0">
+        <v>0</v>
       </c>
       <c r="R198" s="0" t="s">
         <v>25</v>
@@ -14463,7 +14463,7 @@
         <v>46198.89733796296</v>
       </c>
       <c r="F199" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G199" s="0" t="s">
         <v>28</v>
@@ -14531,7 +14531,7 @@
         <v>46213.282858796294</v>
       </c>
       <c r="F200" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G200" s="0" t="s">
         <v>28</v>
@@ -14599,7 +14599,7 @@
         <v>46205.19603009259</v>
       </c>
       <c r="F201" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G201" s="0" t="s">
         <v>28</v>
@@ -14667,7 +14667,7 @@
         <v>46196.08101851852</v>
       </c>
       <c r="F202" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G202" s="0" t="s">
         <v>24</v>
@@ -14735,7 +14735,7 @@
         <v>46196.88885416667</v>
       </c>
       <c r="F203" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G203" s="0" t="s">
         <v>24</v>
@@ -14750,7 +14750,7 @@
         <v>24</v>
       </c>
       <c r="K203" s="0" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="L203" s="0" t="s">
         <v>25</v>
@@ -14770,8 +14770,8 @@
       <c r="Q203" s="0">
         <v>1</v>
       </c>
-      <c r="R203" s="0" t="s">
-        <v>25</v>
+      <c r="R203" s="0">
+        <v>0</v>
       </c>
       <c r="S203" s="0" t="s">
         <v>25</v>
@@ -14803,7 +14803,7 @@
         <v>46199.89765046296</v>
       </c>
       <c r="F204" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G204" s="0" t="s">
         <v>28</v>
@@ -14818,7 +14818,7 @@
         <v>28</v>
       </c>
       <c r="K204" s="0" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="L204" s="0" t="s">
         <v>25</v>
@@ -14838,8 +14838,8 @@
       <c r="Q204" s="0">
         <v>1</v>
       </c>
-      <c r="R204" s="0" t="s">
-        <v>25</v>
+      <c r="R204" s="0">
+        <v>0</v>
       </c>
       <c r="S204" s="0" t="s">
         <v>25</v>
@@ -14871,7 +14871,7 @@
         <v>46203.38673611111</v>
       </c>
       <c r="F205" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G205" s="0" t="s">
         <v>24</v>
@@ -14939,7 +14939,7 @@
         <v>46214.55940972222</v>
       </c>
       <c r="F206" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G206" s="0" t="s">
         <v>28</v>
@@ -15007,7 +15007,7 @@
         <v>46215.391805555555</v>
       </c>
       <c r="F207" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G207" s="0" t="s">
         <v>45</v>
@@ -15075,7 +15075,7 @@
         <v>46208.49730324074</v>
       </c>
       <c r="F208" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G208" s="0" t="s">
         <v>45</v>
@@ -15143,7 +15143,7 @@
         <v>46205.35525462963</v>
       </c>
       <c r="F209" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G209" s="0" t="s">
         <v>28</v>
@@ -15211,7 +15211,7 @@
         <v>46200.595925925925</v>
       </c>
       <c r="F210" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G210" s="0" t="s">
         <v>24</v>
@@ -15279,7 +15279,7 @@
         <v>46198.36408564815</v>
       </c>
       <c r="F211" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G211" s="0" t="s">
         <v>28</v>
@@ -15347,7 +15347,7 @@
         <v>46214.184386574074</v>
       </c>
       <c r="F212" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G212" s="0" t="s">
         <v>28</v>
@@ -15415,7 +15415,7 @@
         <v>46208.95462962963</v>
       </c>
       <c r="F213" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G213" s="0" t="s">
         <v>45</v>
@@ -15483,7 +15483,7 @@
         <v>46209.34474537037</v>
       </c>
       <c r="F214" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G214" s="0" t="s">
         <v>28</v>
@@ -15551,7 +15551,7 @@
         <v>46203.6659375</v>
       </c>
       <c r="F215" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G215" s="0" t="s">
         <v>24</v>
@@ -15563,7 +15563,7 @@
         <v>24</v>
       </c>
       <c r="J215" s="0" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="K215" s="0" t="s">
         <v>25</v>
@@ -15583,8 +15583,8 @@
       <c r="P215" s="0">
         <v>1</v>
       </c>
-      <c r="Q215" s="0" t="s">
-        <v>25</v>
+      <c r="Q215" s="0">
+        <v>0</v>
       </c>
       <c r="R215" s="0" t="s">
         <v>25</v>
@@ -15619,7 +15619,7 @@
         <v>46204.815416666665</v>
       </c>
       <c r="F216" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G216" s="0" t="s">
         <v>24</v>
@@ -15628,7 +15628,7 @@
         <v>24</v>
       </c>
       <c r="I216" s="0" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="J216" s="0" t="s">
         <v>25</v>
@@ -15648,8 +15648,8 @@
       <c r="O216" s="0">
         <v>0</v>
       </c>
-      <c r="P216" s="0" t="s">
-        <v>25</v>
+      <c r="P216" s="0">
+        <v>1</v>
       </c>
       <c r="Q216" s="0" t="s">
         <v>25</v>
@@ -15687,7 +15687,7 @@
         <v>46200.84137731481</v>
       </c>
       <c r="F217" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G217" s="0" t="s">
         <v>28</v>
@@ -15755,7 +15755,7 @@
         <v>46204.81548611111</v>
       </c>
       <c r="F218" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G218" s="0" t="s">
         <v>24</v>
@@ -15764,7 +15764,7 @@
         <v>24</v>
       </c>
       <c r="I218" s="0" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="J218" s="0" t="s">
         <v>25</v>
@@ -15784,8 +15784,8 @@
       <c r="O218" s="0">
         <v>0</v>
       </c>
-      <c r="P218" s="0" t="s">
-        <v>25</v>
+      <c r="P218" s="0">
+        <v>1</v>
       </c>
       <c r="Q218" s="0" t="s">
         <v>25</v>
@@ -15823,7 +15823,7 @@
         <v>46207.322233796294</v>
       </c>
       <c r="F219" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G219" s="0" t="s">
         <v>28</v>
@@ -15835,7 +15835,7 @@
         <v>28</v>
       </c>
       <c r="J219" s="0" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="K219" s="0" t="s">
         <v>25</v>
@@ -15855,8 +15855,8 @@
       <c r="P219" s="0">
         <v>1</v>
       </c>
-      <c r="Q219" s="0" t="s">
-        <v>25</v>
+      <c r="Q219" s="0">
+        <v>0</v>
       </c>
       <c r="R219" s="0" t="s">
         <v>25</v>
@@ -15891,7 +15891,7 @@
         <v>46203.665925925925</v>
       </c>
       <c r="F220" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G220" s="0" t="s">
         <v>24</v>
@@ -15903,7 +15903,7 @@
         <v>24</v>
       </c>
       <c r="J220" s="0" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="K220" s="0" t="s">
         <v>25</v>
@@ -15923,8 +15923,8 @@
       <c r="P220" s="0">
         <v>1</v>
       </c>
-      <c r="Q220" s="0" t="s">
-        <v>25</v>
+      <c r="Q220" s="0">
+        <v>0</v>
       </c>
       <c r="R220" s="0" t="s">
         <v>25</v>
@@ -15959,7 +15959,7 @@
         <v>46208.80619212963</v>
       </c>
       <c r="F221" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G221" s="0" t="s">
         <v>28</v>
@@ -16027,7 +16027,7 @@
         <v>46207.24060185185</v>
       </c>
       <c r="F222" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G222" s="0" t="s">
         <v>24</v>
@@ -16039,7 +16039,7 @@
         <v>24</v>
       </c>
       <c r="J222" s="0" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="K222" s="0" t="s">
         <v>25</v>
@@ -16059,8 +16059,8 @@
       <c r="P222" s="0">
         <v>1</v>
       </c>
-      <c r="Q222" s="0" t="s">
-        <v>25</v>
+      <c r="Q222" s="0">
+        <v>0</v>
       </c>
       <c r="R222" s="0" t="s">
         <v>25</v>
@@ -16095,7 +16095,7 @@
         <v>46213.36528935185</v>
       </c>
       <c r="F223" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G223" s="0" t="s">
         <v>45</v>
@@ -16163,7 +16163,7 @@
         <v>46202.50537037037</v>
       </c>
       <c r="F224" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G224" s="0" t="s">
         <v>28</v>
@@ -16231,7 +16231,7 @@
         <v>46196.08100694444</v>
       </c>
       <c r="F225" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G225" s="0" t="s">
         <v>45</v>
@@ -16299,7 +16299,7 @@
         <v>46200.24690972222</v>
       </c>
       <c r="F226" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G226" s="0" t="s">
         <v>45</v>
@@ -16335,7 +16335,7 @@
         <v>1</v>
       </c>
       <c r="R226" s="0">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S226" s="0" t="s">
         <v>25</v>
@@ -16367,7 +16367,7 @@
         <v>46200.39493055556</v>
       </c>
       <c r="F227" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G227" s="0" t="s">
         <v>24</v>
@@ -16435,7 +16435,7 @@
         <v>46200.50178240741</v>
       </c>
       <c r="F228" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G228" s="0" t="s">
         <v>28</v>
@@ -16503,7 +16503,7 @@
         <v>46201.81197916667</v>
       </c>
       <c r="F229" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G229" s="0" t="s">
         <v>28</v>
@@ -16518,7 +16518,7 @@
         <v>28</v>
       </c>
       <c r="K229" s="0" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="L229" s="0" t="s">
         <v>25</v>
@@ -16538,8 +16538,8 @@
       <c r="Q229" s="0">
         <v>0</v>
       </c>
-      <c r="R229" s="0" t="s">
-        <v>25</v>
+      <c r="R229" s="0">
+        <v>0</v>
       </c>
       <c r="S229" s="0" t="s">
         <v>25</v>
@@ -16571,7 +16571,7 @@
         <v>46196.87100694444</v>
       </c>
       <c r="F230" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G230" s="0" t="s">
         <v>28</v>
@@ -16639,7 +16639,7 @@
         <v>46211.287673611114</v>
       </c>
       <c r="F231" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G231" s="0" t="s">
         <v>28</v>
@@ -16707,7 +16707,7 @@
         <v>46213.33634259259</v>
       </c>
       <c r="F232" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G232" s="0" t="s">
         <v>28</v>
@@ -16775,7 +16775,7 @@
         <v>46203.38674768519</v>
       </c>
       <c r="F233" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G233" s="0" t="s">
         <v>24</v>
@@ -16843,7 +16843,7 @@
         <v>46199.38827546296</v>
       </c>
       <c r="F234" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G234" s="0" t="s">
         <v>24</v>
@@ -16858,7 +16858,7 @@
         <v>24</v>
       </c>
       <c r="K234" s="0" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="L234" s="0" t="s">
         <v>25</v>
@@ -16878,8 +16878,8 @@
       <c r="Q234" s="0">
         <v>1</v>
       </c>
-      <c r="R234" s="0" t="s">
-        <v>25</v>
+      <c r="R234" s="0">
+        <v>0</v>
       </c>
       <c r="S234" s="0" t="s">
         <v>25</v>
@@ -16911,7 +16911,7 @@
         <v>46211.747569444444</v>
       </c>
       <c r="F235" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G235" s="0" t="s">
         <v>24</v>
@@ -16920,7 +16920,7 @@
         <v>24</v>
       </c>
       <c r="I235" s="0" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="J235" s="0" t="s">
         <v>25</v>
@@ -16940,8 +16940,8 @@
       <c r="O235" s="0">
         <v>0</v>
       </c>
-      <c r="P235" s="0" t="s">
-        <v>25</v>
+      <c r="P235" s="0">
+        <v>1</v>
       </c>
       <c r="Q235" s="0" t="s">
         <v>25</v>
@@ -16979,7 +16979,7 @@
         <v>46214.036574074074</v>
       </c>
       <c r="F236" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G236" s="0" t="s">
         <v>24</v>
@@ -17047,7 +17047,7 @@
         <v>46198.75832175926</v>
       </c>
       <c r="F237" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G237" s="0" t="s">
         <v>24</v>
@@ -17059,7 +17059,7 @@
         <v>24</v>
       </c>
       <c r="J237" s="0" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="K237" s="0" t="s">
         <v>25</v>
@@ -17079,8 +17079,8 @@
       <c r="P237" s="0">
         <v>1</v>
       </c>
-      <c r="Q237" s="0" t="s">
-        <v>25</v>
+      <c r="Q237" s="0">
+        <v>0</v>
       </c>
       <c r="R237" s="0" t="s">
         <v>25</v>
@@ -17115,7 +17115,7 @@
         <v>46213.1378125</v>
       </c>
       <c r="F238" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G238" s="0" t="s">
         <v>28</v>
@@ -17183,7 +17183,7 @@
         <v>46200.08666666667</v>
       </c>
       <c r="F239" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G239" s="0" t="s">
         <v>28</v>
@@ -17198,7 +17198,7 @@
         <v>28</v>
       </c>
       <c r="K239" s="0" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="L239" s="0" t="s">
         <v>25</v>
@@ -17218,8 +17218,8 @@
       <c r="Q239" s="0">
         <v>0</v>
       </c>
-      <c r="R239" s="0" t="s">
-        <v>25</v>
+      <c r="R239" s="0">
+        <v>0</v>
       </c>
       <c r="S239" s="0" t="s">
         <v>25</v>
@@ -17251,7 +17251,7 @@
         <v>46191.20039351852</v>
       </c>
       <c r="F240" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G240" s="0" t="s">
         <v>24</v>
@@ -17319,7 +17319,7 @@
         <v>46198.06826388889</v>
       </c>
       <c r="F241" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G241" s="0" t="s">
         <v>24</v>
@@ -17331,7 +17331,7 @@
         <v>24</v>
       </c>
       <c r="J241" s="0" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="K241" s="0" t="s">
         <v>25</v>
@@ -17351,8 +17351,8 @@
       <c r="P241" s="0">
         <v>1</v>
       </c>
-      <c r="Q241" s="0" t="s">
-        <v>25</v>
+      <c r="Q241" s="0">
+        <v>0</v>
       </c>
       <c r="R241" s="0" t="s">
         <v>25</v>
@@ -17387,7 +17387,7 @@
         <v>46197.6375462963</v>
       </c>
       <c r="F242" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G242" s="0" t="s">
         <v>24</v>
@@ -17455,7 +17455,7 @@
         <v>46197.037523148145</v>
       </c>
       <c r="F243" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G243" s="0" t="s">
         <v>24</v>
@@ -17523,7 +17523,7 @@
         <v>46198.31060185185</v>
       </c>
       <c r="F244" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G244" s="0" t="s">
         <v>28</v>
@@ -17591,7 +17591,7 @@
         <v>46209.31466435185</v>
       </c>
       <c r="F245" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G245" s="0" t="s">
         <v>28</v>
@@ -17659,7 +17659,7 @@
         <v>46206.72038194445</v>
       </c>
       <c r="F246" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G246" s="0" t="s">
         <v>28</v>
@@ -17671,7 +17671,7 @@
         <v>28</v>
       </c>
       <c r="J246" s="0" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="K246" s="0" t="s">
         <v>25</v>
@@ -17691,8 +17691,8 @@
       <c r="P246" s="0">
         <v>1</v>
       </c>
-      <c r="Q246" s="0" t="s">
-        <v>25</v>
+      <c r="Q246" s="0">
+        <v>0</v>
       </c>
       <c r="R246" s="0" t="s">
         <v>25</v>
@@ -17727,7 +17727,7 @@
         <v>46197.46810185185</v>
       </c>
       <c r="F247" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G247" s="0" t="s">
         <v>24</v>
@@ -17763,7 +17763,7 @@
         <v>1</v>
       </c>
       <c r="R247" s="0">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S247" s="0" t="s">
         <v>25</v>
@@ -17795,7 +17795,7 @@
         <v>46202.349328703705</v>
       </c>
       <c r="F248" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G248" s="0" t="s">
         <v>28</v>
@@ -17810,7 +17810,7 @@
         <v>28</v>
       </c>
       <c r="K248" s="0" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="L248" s="0" t="s">
         <v>25</v>
@@ -17830,8 +17830,8 @@
       <c r="Q248" s="0">
         <v>1</v>
       </c>
-      <c r="R248" s="0" t="s">
-        <v>25</v>
+      <c r="R248" s="0">
+        <v>0</v>
       </c>
       <c r="S248" s="0" t="s">
         <v>25</v>
@@ -17863,7 +17863,7 @@
         <v>46198.75665509259</v>
       </c>
       <c r="F249" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G249" s="0" t="s">
         <v>24</v>
@@ -17875,7 +17875,7 @@
         <v>24</v>
       </c>
       <c r="J249" s="0" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="K249" s="0" t="s">
         <v>25</v>
@@ -17895,8 +17895,8 @@
       <c r="P249" s="0">
         <v>1</v>
       </c>
-      <c r="Q249" s="0" t="s">
-        <v>25</v>
+      <c r="Q249" s="0">
+        <v>0</v>
       </c>
       <c r="R249" s="0" t="s">
         <v>25</v>
@@ -17931,7 +17931,7 @@
         <v>46205.784363425926</v>
       </c>
       <c r="F250" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G250" s="0" t="s">
         <v>45</v>
@@ -17943,7 +17943,7 @@
         <v>45</v>
       </c>
       <c r="J250" s="0" t="s">
-        <v>25</v>
+        <v>45</v>
       </c>
       <c r="K250" s="0" t="s">
         <v>25</v>
@@ -17963,8 +17963,8 @@
       <c r="P250" s="0">
         <v>1</v>
       </c>
-      <c r="Q250" s="0" t="s">
-        <v>25</v>
+      <c r="Q250" s="0">
+        <v>0</v>
       </c>
       <c r="R250" s="0" t="s">
         <v>25</v>
@@ -17999,7 +17999,7 @@
         <v>46204.81548611111</v>
       </c>
       <c r="F251" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G251" s="0" t="s">
         <v>24</v>
@@ -18008,7 +18008,7 @@
         <v>24</v>
       </c>
       <c r="I251" s="0" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="J251" s="0" t="s">
         <v>25</v>
@@ -18028,8 +18028,8 @@
       <c r="O251" s="0">
         <v>0</v>
       </c>
-      <c r="P251" s="0" t="s">
-        <v>25</v>
+      <c r="P251" s="0">
+        <v>1</v>
       </c>
       <c r="Q251" s="0" t="s">
         <v>25</v>
@@ -18067,7 +18067,7 @@
         <v>46204.81548611111</v>
       </c>
       <c r="F252" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G252" s="0" t="s">
         <v>24</v>
@@ -18076,7 +18076,7 @@
         <v>24</v>
       </c>
       <c r="I252" s="0" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="J252" s="0" t="s">
         <v>25</v>
@@ -18096,8 +18096,8 @@
       <c r="O252" s="0">
         <v>0</v>
       </c>
-      <c r="P252" s="0" t="s">
-        <v>25</v>
+      <c r="P252" s="0">
+        <v>1</v>
       </c>
       <c r="Q252" s="0" t="s">
         <v>25</v>
@@ -18135,7 +18135,7 @@
         <v>46198.75827546296</v>
       </c>
       <c r="F253" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G253" s="0" t="s">
         <v>24</v>
@@ -18147,7 +18147,7 @@
         <v>24</v>
       </c>
       <c r="J253" s="0" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="K253" s="0" t="s">
         <v>25</v>
@@ -18167,8 +18167,8 @@
       <c r="P253" s="0">
         <v>1</v>
       </c>
-      <c r="Q253" s="0" t="s">
-        <v>25</v>
+      <c r="Q253" s="0">
+        <v>0</v>
       </c>
       <c r="R253" s="0" t="s">
         <v>25</v>
@@ -18203,7 +18203,7 @@
         <v>46203.80048611111</v>
       </c>
       <c r="F254" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G254" s="0" t="s">
         <v>45</v>
@@ -18271,7 +18271,7 @@
         <v>46207.377118055556</v>
       </c>
       <c r="F255" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G255" s="0" t="s">
         <v>28</v>
@@ -18283,7 +18283,7 @@
         <v>28</v>
       </c>
       <c r="J255" s="0" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="K255" s="0" t="s">
         <v>25</v>
@@ -18303,8 +18303,8 @@
       <c r="P255" s="0">
         <v>0</v>
       </c>
-      <c r="Q255" s="0" t="s">
-        <v>25</v>
+      <c r="Q255" s="0">
+        <v>0</v>
       </c>
       <c r="R255" s="0" t="s">
         <v>25</v>
@@ -18339,7 +18339,7 @@
         <v>46198.76320601852</v>
       </c>
       <c r="F256" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G256" s="0" t="s">
         <v>24</v>
@@ -18351,7 +18351,7 @@
         <v>24</v>
       </c>
       <c r="J256" s="0" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="K256" s="0" t="s">
         <v>25</v>
@@ -18371,8 +18371,8 @@
       <c r="P256" s="0">
         <v>1</v>
       </c>
-      <c r="Q256" s="0" t="s">
-        <v>25</v>
+      <c r="Q256" s="0">
+        <v>0</v>
       </c>
       <c r="R256" s="0" t="s">
         <v>25</v>
@@ -18407,7 +18407,7 @@
         <v>46209.364849537036</v>
       </c>
       <c r="F257" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G257" s="0" t="s">
         <v>45</v>
@@ -18475,7 +18475,7 @@
         <v>46198.76327546296</v>
       </c>
       <c r="F258" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G258" s="0" t="s">
         <v>24</v>
@@ -18487,7 +18487,7 @@
         <v>24</v>
       </c>
       <c r="J258" s="0" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="K258" s="0" t="s">
         <v>25</v>
@@ -18507,8 +18507,8 @@
       <c r="P258" s="0">
         <v>1</v>
       </c>
-      <c r="Q258" s="0" t="s">
-        <v>25</v>
+      <c r="Q258" s="0">
+        <v>0</v>
       </c>
       <c r="R258" s="0" t="s">
         <v>25</v>
@@ -18543,7 +18543,7 @@
         <v>46197.041238425925</v>
       </c>
       <c r="F259" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G259" s="0" t="s">
         <v>24</v>
@@ -18611,7 +18611,7 @@
         <v>46212.017488425925</v>
       </c>
       <c r="F260" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G260" s="0" t="s">
         <v>45</v>
@@ -18679,7 +18679,7 @@
         <v>46204.81549768519</v>
       </c>
       <c r="F261" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G261" s="0" t="s">
         <v>24</v>
@@ -18688,7 +18688,7 @@
         <v>24</v>
       </c>
       <c r="I261" s="0" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="J261" s="0" t="s">
         <v>25</v>
@@ -18708,8 +18708,8 @@
       <c r="O261" s="0">
         <v>0</v>
       </c>
-      <c r="P261" s="0" t="s">
-        <v>25</v>
+      <c r="P261" s="0">
+        <v>1</v>
       </c>
       <c r="Q261" s="0" t="s">
         <v>25</v>
@@ -18747,7 +18747,7 @@
         <v>46200.44310185185</v>
       </c>
       <c r="F262" s="1">
-        <v>46216.04230405093</v>
+        <v>46217.042329282405</v>
       </c>
       <c r="G262" s="0" t="s">
         <v>24</v>

</xml_diff>